<commit_message>
Pruebas del Sprint 3 completo: programaciones, terceros, procedimientos y permisos con evidencia
- Informe de Pruebas S3 de todo el sprint (64 casos, 55 ok); HU-151 pasa al
  manifiesto de S6.
- BD/241: la OT generada desde una ocurrencia trae un paso por cada paso del
  procedimiento, con el texto copiado (HU-062 #1, HU-061 #2).
- BD/242: tomar una OT con permisos vencidos se rechaza (HU-063 #3); consumo
  contra OT de repuesto no compatible exige motivo (HU-051 #2).
- Backlog S3: criterios marcados, tareas de pruebas terminadas, historias
  observadas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S3.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S3.xlsx
@@ -2335,10 +2335,14 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="O7" s="11" t="n"/>
+      <c r="O7" s="11" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="P7" s="11" t="inlineStr">
         <is>
-          <t>DECISIÓN TOMADA 12-09-2026 (Bryan): pme_activo_medidor pasa a NULL (BD/224). Con NULL, el medidor lo aporta cada equipo del plan (Plan_Mantenimiento_Activo.pac_activo_medidor, HU-083). Una programación, cuatro blowers. Falta el disparo por lectura (generador por medidor).</t>
+          <t>Pruebas S3 (17-09): #3 OK (medidor por equipo). #1/#2 NO: el disparo por lectura no está construido (pendiente §10.9). DECISIÓN TOMADA 12-09-2026 (Bryan): pme_activo_medidor pasa a NULL (BD/224). Con NULL, el medidor lo aporta cada equipo del plan (Plan_Mantenimiento_Activo.pac_activo_medidor, HU-083). Una programación, cuatro blowers. Falta el disparo por lectura (generador por medidor).</t>
         </is>
       </c>
     </row>
@@ -2481,10 +2485,14 @@
           <t>En revisión</t>
         </is>
       </c>
-      <c r="O9" s="11" t="n"/>
+      <c r="O9" s="11" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="P9" s="11" t="inlineStr">
         <is>
-          <t>Base de datos y web terminadas. El último día del mes y el último viernes salen correctos, incluido febrero bisiesto.</t>
+          <t>Pruebas S3 (17-09): 3 criterios OK (martes/jueves, último día del mes con bisiesto, último viernes). Base de datos y web terminadas. El último día del mes y el último viernes salen correctos, incluido febrero bisiesto.</t>
         </is>
       </c>
     </row>
@@ -2852,10 +2860,14 @@
           <t>En revisión</t>
         </is>
       </c>
-      <c r="O14" s="7" t="n"/>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>Base de datos y web terminadas. Hizo falta agregar pxc_desplaza para separar la parada de planta (no genera) del feriado (corre la fecha y guarda la original).</t>
+          <t>Pruebas S3 (17-09): 3 criterios OK (ventana, feriado desplazado con fecha original, parada de planta). Base de datos y web terminadas. Hizo falta agregar pxc_desplaza para separar la parada de planta (no genera) del feriado (corre la fecha y guarda la original).</t>
         </is>
       </c>
     </row>
@@ -2995,11 +3007,19 @@
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="O16" s="7" t="n"/>
-      <c r="P16" s="7" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="O16" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="P16" s="7" t="inlineStr">
+        <is>
+          <t>Construida por Bryan (bloque 91). Pruebas S3 (17-09): 2 criterios OK.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="54.75" customHeight="1" s="19">
       <c r="A17" s="9" t="inlineStr">
@@ -3062,11 +3082,19 @@
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="O17" s="11" t="n"/>
-      <c r="P17" s="11" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="O17" s="11" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="P17" s="11" t="inlineStr">
+        <is>
+          <t>Construida por Bryan (bloque 92). Pruebas S3 (17-09): #1 OK; #2 OK con la regla nueva del bloque 242 (consumo contra OT de un equipo no compatible exige el motivo).</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="54.75" customHeight="1" s="19">
       <c r="A18" s="6" t="inlineStr">
@@ -3289,7 +3317,7 @@
       </c>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>Construida por Emilio Fuentes (01-09-2026). La BD ya estaba (bloque 101: SEL/INS/UPD/DEL_PROCEDIMIENTO y SEL_VARIABLE_MEDICION); revisada y confirmada. AGREGADO: datos de prueba (bloque 130), pantallas en Mantenimiento → Procedimientos (listado + ficha, patrón SigmaModal, ficha rediseñada estilo Programaciones) y permisos/menú (bloque 131). El código no es automático a propósito: la llave es (cliente, código, versión). Compila exitcode=0. PENDIENTE: prueba en navegador (verificación de criterios, de Catalina).</t>
+          <t>Pruebas S3 (17-09): 2 criterios OK; la OT generada copia los pasos del procedimiento (bloque 241). Construida por Emilio Fuentes (01-09-2026). La BD ya estaba (bloque 101: SEL/INS/UPD/DEL_PROCEDIMIENTO y SEL_VARIABLE_MEDICION); revisada y confirmada. AGREGADO: datos de prueba (bloque 130), pantallas en Mantenimiento → Procedimientos (listado + ficha, patrón SigmaModal, ficha rediseñada estilo Programaciones) y permisos/menú (bloque 131). El código no es automático a propósito: la llave es (cliente, código, versión). Compila exitcode=0. PENDIENTE: prueba en navegador (verificación de criterios, de Catalina).</t>
         </is>
       </c>
     </row>
@@ -3354,11 +3382,19 @@
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="O21" s="11" t="n"/>
-      <c r="P21" s="11" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="O21" s="11" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="P21" s="11" t="inlineStr">
+        <is>
+          <t>Construida por Bryan (bloque 94). Pruebas S3 (17-09): #1 y #2 OK (el documento firmado es obligatorio para autorizar; la subida depende de la API de archivos del Sprint 6); #3 OK con la regla nueva del bloque 242 (tomar la OT con el permiso vencido se rechaza).</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="82.5" customHeight="1" s="19">
       <c r="A22" s="6" t="inlineStr">
@@ -3424,10 +3460,14 @@
           <t>En revisión</t>
         </is>
       </c>
-      <c r="O22" s="7" t="n"/>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>Base de datos y web terminadas. Los criterios se pueden ejercitar con la vista previa de fechas de la ficha.</t>
+          <t>Pruebas S3 (17-09): 2 criterios OK sobre FNC_PROGRAMACION_FECHAS y la ficha. Base de datos y web terminadas. Los criterios se pueden ejercitar con la vista previa de fechas de la ficha.</t>
         </is>
       </c>
     </row>
@@ -3495,10 +3535,14 @@
           <t>En revisión</t>
         </is>
       </c>
-      <c r="O23" s="11" t="n"/>
+      <c r="O23" s="11" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="P23" s="11" t="inlineStr">
         <is>
-          <t>Base de datos y web terminadas. Hizo falta agregar pin_desde_ejecucion: sin esa columna los dos criterios de la historia se contradicen.</t>
+          <t>Pruebas S3 (17-09): 2 criterios OK. Base de datos y web terminadas. Hizo falta agregar pin_desde_ejecucion: sin esa columna los dos criterios de la historia se contradicen.</t>
         </is>
       </c>
     </row>
@@ -3566,10 +3610,14 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="O24" s="7" t="n"/>
+      <c r="O24" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>DESBLOQUEADA 12-09-2026: HU-041 cerrada por Bryan (BD/224) y datos de prueba cargados (T-3261). El combo de variables ya tiene opciones.</t>
+          <t>Pruebas S3 (17-09): #1-#3 NO: las condiciones se definen pero el disparo al registrar la medición no está construido (pendiente §10.9). DESBLOQUEADA 12-09-2026: HU-041 cerrada por Bryan (BD/224) y datos de prueba cargados (T-3261). El combo de variables ya tiene opciones.</t>
         </is>
       </c>
     </row>
@@ -3719,7 +3767,7 @@
       </c>
       <c r="P26" s="10" t="inlineStr">
         <is>
-          <t>Construida por Emilio Fuentes (06-09-2026): BD (SEL/INS/UPD/DEL_PROCEDIMIENTO_PASO en BD/156, con orden unico por procedimiento, medicion que exige variable y baja logica que respeta ordenes) + Web (listado ProcedimientoPasos y ficha ProcedimientoPaso, con modelo/controller ProcedimientoPaso y VariableMedicion) + Menus (BD/157) + seguridad por cliente. Datos de prueba: los 10 pasos del procedimiento CAMBIO-MOTORREDUCTOR (BD/155). PENDIENTE (otra persona): pruebas por criterio, documentacion/Swagger y consumo movil.</t>
+          <t>Pruebas S3 (17-09): #1 OK (bloque 241: un paso de OT por cada paso del procedimiento); #2 y #3 quedan definidos en la web y su exigencia al ejecutar es de la app (Sprint 6). Construida por Emilio Fuentes (06-09-2026): BD (SEL/INS/UPD/DEL_PROCEDIMIENTO_PASO en BD/156, con orden unico por procedimiento, medicion que exige variable y baja logica que respeta ordenes) + Web (listado ProcedimientoPasos y ficha ProcedimientoPaso, con modelo/controller ProcedimientoPaso y VariableMedicion) + Menus (BD/157) + seguridad por cliente. Datos de prueba: los 10 pasos del procedimiento CAMBIO-MOTORREDUCTOR (BD/155). PENDIENTE (otra persona): pruebas por criterio, documentacion/Swagger y consumo movil.</t>
         </is>
       </c>
     </row>
@@ -3859,13 +3907,17 @@
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="O28" s="7" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="O28" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
       <c r="P28" s="7" t="inlineStr">
         <is>
-          <t>· ALCANCE APP (30-08): Web → Web y App. Promovida a App: el prevencionista verifica el permiso en el frente de trabajo.</t>
+          <t>Construida por Bryan (bloque 97). Pruebas S3 (17-09): 2 criterios OK. · ALCANCE APP (30-08): Web → Web y App. Promovida a App: el prevencionista verifica el permiso en el frente de trabajo.</t>
         </is>
       </c>
     </row>
@@ -6503,11 +6555,17 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="n"/>
-      <c r="J28" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="27" customHeight="1" s="19">
       <c r="A29" s="6" t="inlineStr">
@@ -7569,11 +7627,17 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I51" s="6" t="n"/>
-      <c r="J51" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="41.25" customHeight="1" s="19">
       <c r="A52" s="6" t="inlineStr">
@@ -8175,11 +8239,17 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I64" s="6" t="n"/>
-      <c r="J64" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="41.25" customHeight="1" s="19">
       <c r="A65" s="6" t="inlineStr">
@@ -8833,11 +8903,17 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I78" s="6" t="n"/>
-      <c r="J78" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="27" customHeight="1" s="19">
       <c r="A79" s="6" t="inlineStr">
@@ -9397,11 +9473,17 @@
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I90" s="6" t="n"/>
-      <c r="J90" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I90" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J90" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="27" customHeight="1" s="19">
       <c r="A91" s="6" t="inlineStr">
@@ -9911,11 +9993,17 @@
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I101" s="6" t="n"/>
-      <c r="J101" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I101" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J101" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="27" customHeight="1" s="19">
       <c r="A102" s="6" t="inlineStr">
@@ -10455,11 +10543,17 @@
       </c>
       <c r="H113" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I113" s="6" t="n"/>
-      <c r="J113" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I113" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J113" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="41.25" customHeight="1" s="19">
       <c r="A114" s="6" t="inlineStr">
@@ -11113,11 +11207,17 @@
       </c>
       <c r="H127" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I127" s="6" t="n"/>
-      <c r="J127" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I127" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J127" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="27" customHeight="1" s="19">
       <c r="A128" s="6" t="inlineStr">
@@ -11617,11 +11717,17 @@
       </c>
       <c r="H139" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I139" s="6" t="n"/>
-      <c r="J139" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I139" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J139" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="27" customHeight="1" s="19">
       <c r="A140" s="6" t="inlineStr">
@@ -12121,11 +12227,17 @@
       </c>
       <c r="H151" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I151" s="6" t="n"/>
-      <c r="J151" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I151" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J151" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="27" customHeight="1" s="19">
       <c r="A152" s="6" t="inlineStr">
@@ -12685,11 +12797,17 @@
       </c>
       <c r="H163" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I163" s="6" t="n"/>
-      <c r="J163" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I163" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J163" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="41.25" customHeight="1" s="19">
       <c r="A164" s="6" t="inlineStr">
@@ -13057,11 +13175,17 @@
       </c>
       <c r="H171" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I171" s="6" t="n"/>
-      <c r="J171" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I171" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J171" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="41.25" customHeight="1" s="19">
       <c r="A172" s="6" t="inlineStr">
@@ -13601,11 +13725,17 @@
       </c>
       <c r="H183" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I183" s="6" t="n"/>
-      <c r="J183" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I183" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J183" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="184" hidden="1" ht="27" customHeight="1" s="19">
       <c r="A184" s="6" t="inlineStr">
@@ -14193,11 +14323,17 @@
       </c>
       <c r="H197" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I197" s="6" t="n"/>
-      <c r="J197" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I197" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J197" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="198" ht="27" customHeight="1" s="19">
       <c r="A198" s="6" t="inlineStr">
@@ -14645,11 +14781,17 @@
       </c>
       <c r="H207" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I207" s="6" t="n"/>
-      <c r="J207" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I207" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J207" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="208" ht="41.25" customHeight="1" s="19">
       <c r="A208" s="6" t="inlineStr">
@@ -15097,11 +15239,17 @@
       </c>
       <c r="H217" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I217" s="6" t="n"/>
-      <c r="J217" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I217" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J217" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="218" ht="27" customHeight="1" s="19">
       <c r="A218" s="6" t="inlineStr">
@@ -15551,11 +15699,17 @@
       </c>
       <c r="H227" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I227" s="6" t="n"/>
-      <c r="J227" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I227" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J227" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="228" ht="27" customHeight="1" s="19">
       <c r="A228" s="6" t="inlineStr">
@@ -16163,11 +16317,17 @@
       </c>
       <c r="H240" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I240" s="6" t="n"/>
-      <c r="J240" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I240" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J240" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="241" ht="27" customHeight="1" s="19">
       <c r="A241" s="6" t="inlineStr">
@@ -16753,11 +16913,17 @@
       </c>
       <c r="H253" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I253" s="6" t="n"/>
-      <c r="J253" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I253" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J253" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="254" hidden="1" ht="41.25" customHeight="1" s="19">
       <c r="A254" s="6" t="inlineStr">
@@ -17125,11 +17291,17 @@
       </c>
       <c r="H261" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I261" s="6" t="n"/>
-      <c r="J261" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I261" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J261" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="262" ht="27" customHeight="1" s="19">
       <c r="A262" s="6" t="inlineStr">
@@ -17545,11 +17717,17 @@
       </c>
       <c r="H271" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I271" s="6" t="n"/>
-      <c r="J271" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I271" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J271" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="272" ht="54.75" customHeight="1" s="19">
       <c r="A272" s="6" t="inlineStr">
@@ -19705,11 +19883,17 @@
       </c>
       <c r="H322" s="6" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I322" s="6" t="n"/>
-      <c r="J322" s="7" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I322" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J322" s="7" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 3, capturas/S3).</t>
+        </is>
+      </c>
     </row>
     <row r="323" ht="41.25" customHeight="1" s="19">
       <c r="A323" s="6" t="inlineStr">
@@ -21301,7 +21485,7 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -21459,7 +21643,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -21491,7 +21675,7 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -21522,7 +21706,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -21872,7 +22056,7 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -21904,7 +22088,7 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -21935,7 +22119,7 @@
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22032,7 +22216,7 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22064,7 +22248,7 @@
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22095,7 +22279,7 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22126,7 +22310,7 @@
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22315,7 +22499,7 @@
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22347,7 +22531,7 @@
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22379,7 +22563,7 @@
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22410,7 +22594,7 @@
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22442,7 +22626,7 @@
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22505,7 +22689,7 @@
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22537,7 +22721,7 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22568,7 +22752,7 @@
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22758,7 +22942,7 @@
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22917,7 +23101,7 @@
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22948,7 +23132,7 @@
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 3: generacion por medidor y por condicion; paso con medicion y punto de control
- BD/243: FNC_PLAN_MEDIDOR_ESTADO (el horometro de cada equipo del plan y el
  proximo valor), GEN_PLAN_OCURRENCIAS_MEDIDOR (ocurrencia al alcanzar el
  valor, alerta de aviso sin OT) y GEN_PLAN_OCURRENCIAS_CONDICION (racha por
  duracion minima, politica TODOS/UNO). Los SP de captura los llaman tras el
  commit. UPS_PROGRAMACION_MEDIDOR acepta medidor vacio.
- BD/244: API_UPD_ORDEN_TRABAJO_PASO exige la medicion del paso y la registra
  en la serie con la OT como origen; un punto de control pendiente bloquea.
  PasoResultadoDto gana valor_medicion / unidad_medida.
- Evidencia S3 (ev_s3h.py): HU-073 #1-#3, HU-074 #1-#3, HU-062 #2/#3 OK.
  Informe S3 63/64. Backlog S3: tareas T-3972..3977 a Bryan, HU-073/074 en
  revision.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S3.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S3.xlsx
@@ -2252,7 +2252,7 @@
         <v>3</v>
       </c>
       <c r="M6" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A6,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A6,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N6" s="6" t="inlineStr">
@@ -2327,12 +2327,12 @@
         <v>3</v>
       </c>
       <c r="M7" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A7,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A7,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="O7" s="11" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="P7" s="11" t="inlineStr">
         <is>
-          <t>Pruebas S3 (17-09): #3 OK (medidor por equipo). #1/#2 NO: el disparo por lectura no está construido (pendiente §10.9). DECISIÓN TOMADA 12-09-2026 (Bryan): pme_activo_medidor pasa a NULL (BD/224). Con NULL, el medidor lo aporta cada equipo del plan (Plan_Mantenimiento_Activo.pac_activo_medidor, HU-083). Una programación, cuatro blowers. Falta el disparo por lectura (generador por medidor).</t>
+          <t>Tomada por Bryan el 17-09-2026: disparo por lectura/medición construido (bloque 243) y los 3 criterios OK con evidencia. Pruebas S3 (17-09): #3 OK (medidor por equipo). #1/#2 NO: el disparo por lectura no está construido (pendiente §10.9). DECISIÓN TOMADA 12-09-2026 (Bryan): pme_activo_medidor pasa a NULL (BD/224). Con NULL, el medidor lo aporta cada equipo del plan (Plan_Mantenimiento_Activo.pac_activo_medidor, HU-083). Una programación, cuatro blowers. Falta el disparo por lectura (generador por medidor).</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
         <v>4</v>
       </c>
       <c r="M8" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A8,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A8,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N8" s="6" t="inlineStr">
@@ -2477,7 +2477,7 @@
         <v>3</v>
       </c>
       <c r="M9" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A9,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A9,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -2552,7 +2552,7 @@
         <v>3</v>
       </c>
       <c r="M10" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A10,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A10,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N10" s="6" t="inlineStr">
@@ -2627,7 +2627,7 @@
         <v>3</v>
       </c>
       <c r="M11" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A11,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A11,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N11" s="9" t="inlineStr">
@@ -2702,7 +2702,7 @@
         <v>2</v>
       </c>
       <c r="M12" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A12,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A12,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N12" s="6" t="inlineStr">
@@ -2777,7 +2777,7 @@
         <v>2</v>
       </c>
       <c r="M13" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A13,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A13,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N13" s="9" t="inlineStr">
@@ -2852,7 +2852,7 @@
         <v>3</v>
       </c>
       <c r="M14" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A14,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A14,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N14" s="6" t="inlineStr">
@@ -2927,7 +2927,7 @@
         <v>2</v>
       </c>
       <c r="M15" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A15,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A15,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N15" s="9" t="inlineStr">
@@ -3002,7 +3002,7 @@
         <v>2</v>
       </c>
       <c r="M16" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A16,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A16,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N16" s="6" t="inlineStr">
@@ -3077,7 +3077,7 @@
         <v>2</v>
       </c>
       <c r="M17" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A17,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A17,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N17" s="9" t="inlineStr">
@@ -3152,7 +3152,7 @@
         <v>2</v>
       </c>
       <c r="M18" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A18,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A18,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N18" s="6" t="inlineStr">
@@ -3227,7 +3227,7 @@
         <v>3</v>
       </c>
       <c r="M19" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A19,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A19,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N19" s="9" t="inlineStr">
@@ -3302,7 +3302,7 @@
         <v>2</v>
       </c>
       <c r="M20" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A20,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A20,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N20" s="6" t="inlineStr">
@@ -3377,7 +3377,7 @@
         <v>3</v>
       </c>
       <c r="M21" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A21,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A21,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N21" s="9" t="inlineStr">
@@ -3452,7 +3452,7 @@
         <v>2</v>
       </c>
       <c r="M22" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A22,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A22,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N22" s="6" t="inlineStr">
@@ -3527,7 +3527,7 @@
         <v>2</v>
       </c>
       <c r="M23" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A23,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A23,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -3602,12 +3602,12 @@
         <v>3</v>
       </c>
       <c r="M24" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A24,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A24,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="O24" s="7" t="inlineStr">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>Pruebas S3 (17-09): #1-#3 NO: las condiciones se definen pero el disparo al registrar la medición no está construido (pendiente §10.9). DESBLOQUEADA 12-09-2026: HU-041 cerrada por Bryan (BD/224) y datos de prueba cargados (T-3261). El combo de variables ya tiene opciones.</t>
+          <t>Tomada por Bryan el 17-09-2026: disparo por lectura/medición construido (bloque 243) y los 3 criterios OK con evidencia. Pruebas S3 (17-09): #1-#3 NO: las condiciones se definen pero el disparo al registrar la medición no está construido (pendiente §10.9). DESBLOQUEADA 12-09-2026: HU-041 cerrada por Bryan (BD/224) y datos de prueba cargados (T-3261). El combo de variables ya tiene opciones.</t>
         </is>
       </c>
     </row>
@@ -3677,7 +3677,7 @@
         <v>2</v>
       </c>
       <c r="M25" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A25,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A25,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N25" s="9" t="inlineStr">
@@ -3752,7 +3752,7 @@
         <v>3</v>
       </c>
       <c r="M26" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A26,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A26,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N26" s="6" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="P26" s="10" t="inlineStr">
         <is>
-          <t>Pruebas S3 (17-09): #1 OK (bloque 241: un paso de OT por cada paso del procedimiento); #2 y #3 quedan definidos en la web y su exigencia al ejecutar es de la app (Sprint 6). Construida por Emilio Fuentes (06-09-2026): BD (SEL/INS/UPD/DEL_PROCEDIMIENTO_PASO en BD/156, con orden unico por procedimiento, medicion que exige variable y baja logica que respeta ordenes) + Web (listado ProcedimientoPasos y ficha ProcedimientoPaso, con modelo/controller ProcedimientoPaso y VariableMedicion) + Menus (BD/157) + seguridad por cliente. Datos de prueba: los 10 pasos del procedimiento CAMBIO-MOTORREDUCTOR (BD/155). PENDIENTE (otra persona): pruebas por criterio, documentacion/Swagger y consumo movil.</t>
+          <t>Bryan (17-09-2026): el servidor exige la medición y respeta el punto de control al completar el paso (bloque 244); #2 y #3 OK por API. Pruebas S3 (17-09): #1 OK (bloque 241: un paso de OT por cada paso del procedimiento); #2 y #3 quedan definidos en la web y su exigencia al ejecutar es de la app (Sprint 6). Construida por Emilio Fuentes (06-09-2026): BD (SEL/INS/UPD/DEL_PROCEDIMIENTO_PASO en BD/156, con orden unico por procedimiento, medicion que exige variable y baja logica que respeta ordenes) + Web (listado ProcedimientoPasos y ficha ProcedimientoPaso, con modelo/controller ProcedimientoPaso y VariableMedicion) + Menus (BD/157) + seguridad por cliente. Datos de prueba: los 10 pasos del procedimiento CAMBIO-MOTORREDUCTOR (BD/155). PENDIENTE (otra persona): pruebas por criterio, documentacion/Swagger y consumo movil.</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
         <v>2</v>
       </c>
       <c r="M27" s="9">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A27,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A27,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N27" s="9" t="inlineStr">
@@ -3902,7 +3902,7 @@
         <v>2</v>
       </c>
       <c r="M28" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A28,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A28,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N28" s="6" t="inlineStr">
@@ -3977,7 +3977,7 @@
         <v>4</v>
       </c>
       <c r="M29" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A29,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A29,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N29" s="6" t="inlineStr">
@@ -4052,7 +4052,7 @@
         <v>3</v>
       </c>
       <c r="M30" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A30,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A30,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N30" s="6" t="inlineStr">
@@ -4127,7 +4127,7 @@
         <v>3</v>
       </c>
       <c r="M31" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A31,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A31,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N31" s="6" t="inlineStr">
@@ -4202,7 +4202,7 @@
         <v>2</v>
       </c>
       <c r="M32" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A32,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A32,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N32" s="6" t="inlineStr">
@@ -4277,7 +4277,7 @@
         <v>2</v>
       </c>
       <c r="M33" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A33,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A33,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N33" s="6" t="inlineStr">
@@ -4352,7 +4352,7 @@
         <v>4</v>
       </c>
       <c r="M34" s="6">
-        <f>SUMIF(Tareas!$B$6:$B$335,$A34,Tareas!$F$6:$F$335)</f>
+        <f>SUMIF(Tareas!$B$6:$B$341,$A34,Tareas!$F$6:$F$341)</f>
         <v/>
       </c>
       <c r="N34" s="6" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J335"/>
+  <dimension ref="A1:J341"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.7109375" customWidth="1" style="19" min="1" max="1"/>
@@ -20489,12 +20489,294 @@
       </c>
       <c r="J335" s="7" t="n"/>
     </row>
-    <row r="336" ht="15.75" customHeight="1" s="19"/>
-    <row r="337" ht="15.75" customHeight="1" s="19"/>
-    <row r="338" ht="15.75" customHeight="1" s="19"/>
-    <row r="339" ht="15.75" customHeight="1" s="19"/>
-    <row r="340" ht="15.75" customHeight="1" s="19"/>
-    <row r="341" ht="15.75" customHeight="1" s="19"/>
+    <row r="336" ht="15.75" customHeight="1" s="19">
+      <c r="A336" s="6" t="inlineStr">
+        <is>
+          <t>T-3972</t>
+        </is>
+      </c>
+      <c r="B336" s="6" t="inlineStr">
+        <is>
+          <t>HU-073</t>
+        </is>
+      </c>
+      <c r="C336" s="7" t="inlineStr">
+        <is>
+          <t>Crear una programación por medidor</t>
+        </is>
+      </c>
+      <c r="D336" s="10" t="inlineStr">
+        <is>
+          <t>FNC_PLAN_MEDIDOR_ESTADO + GEN_PLAN_OCURRENCIAS_MEDIDOR (bloque 243): el horómetro de cada equipo del plan, próximo valor desde la última ocurrencia, ocurrencia al alcanzarlo (#1/#3) y alerta de aviso sin OT dentro de la anticipación (#2).</t>
+        </is>
+      </c>
+      <c r="E336" s="6" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
+      <c r="F336" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G336" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="H336" s="6" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I336" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J336" s="7" t="inlineStr">
+        <is>
+          <t>Construido y probado el 17-09-2026 (evidencia S3 por criterio). Tomado por Bryan a pedido suyo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="15.75" customHeight="1" s="19">
+      <c r="A337" s="6" t="inlineStr">
+        <is>
+          <t>T-3973</t>
+        </is>
+      </c>
+      <c r="B337" s="6" t="inlineStr">
+        <is>
+          <t>HU-073</t>
+        </is>
+      </c>
+      <c r="C337" s="7" t="inlineStr">
+        <is>
+          <t>Crear una programación por medidor</t>
+        </is>
+      </c>
+      <c r="D337" s="10" t="inlineStr">
+        <is>
+          <t>API_INS_ACTIVO_MEDIDOR_LECTURA llama al generador tras el commit; UPS_PROGRAMACION_MEDIDOR acepta medidor vacío (= el de cada equipo); GEN_ALERTA_OPERACION comparte la vista.</t>
+        </is>
+      </c>
+      <c r="E337" s="6" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
+      <c r="F337" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G337" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="H337" s="6" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I337" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J337" s="7" t="inlineStr">
+        <is>
+          <t>Construido y probado el 17-09-2026 (evidencia S3 por criterio). Tomado por Bryan a pedido suyo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="15.75" customHeight="1" s="19">
+      <c r="A338" s="6" t="inlineStr">
+        <is>
+          <t>T-3974</t>
+        </is>
+      </c>
+      <c r="B338" s="6" t="inlineStr">
+        <is>
+          <t>HU-074</t>
+        </is>
+      </c>
+      <c r="C338" s="7" t="inlineStr">
+        <is>
+          <t>Crear una programación por condición</t>
+        </is>
+      </c>
+      <c r="D338" s="10" t="inlineStr">
+        <is>
+          <t>GEN_PLAN_OCURRENCIAS_CONDICION (bloque 243): evalúa las condiciones sobre la última medición en la unidad de la variable, duración mínima por racha (#2) y política TODOS/UNO (#3); una ocurrencia viva por hito y equipo.</t>
+        </is>
+      </c>
+      <c r="E338" s="6" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
+      <c r="F338" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G338" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="H338" s="6" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I338" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J338" s="7" t="inlineStr">
+        <is>
+          <t>Construido y probado el 17-09-2026 (evidencia S3 por criterio). Tomado por Bryan a pedido suyo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="15.75" customHeight="1" s="19">
+      <c r="A339" s="6" t="inlineStr">
+        <is>
+          <t>T-3975</t>
+        </is>
+      </c>
+      <c r="B339" s="6" t="inlineStr">
+        <is>
+          <t>HU-074</t>
+        </is>
+      </c>
+      <c r="C339" s="7" t="inlineStr">
+        <is>
+          <t>Crear una programación por condición</t>
+        </is>
+      </c>
+      <c r="D339" s="10" t="inlineStr">
+        <is>
+          <t>API_INS_ACTIVO_MEDICION llama al generador tras el commit, con su propio TRY para no perder la medición.</t>
+        </is>
+      </c>
+      <c r="E339" s="6" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
+      <c r="F339" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G339" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="H339" s="6" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I339" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J339" s="7" t="inlineStr">
+        <is>
+          <t>Construido y probado el 17-09-2026 (evidencia S3 por criterio). Tomado por Bryan a pedido suyo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="340" ht="15.75" customHeight="1" s="19">
+      <c r="A340" s="6" t="inlineStr">
+        <is>
+          <t>T-3976</t>
+        </is>
+      </c>
+      <c r="B340" s="6" t="inlineStr">
+        <is>
+          <t>HU-062</t>
+        </is>
+      </c>
+      <c r="C340" s="7" t="inlineStr">
+        <is>
+          <t>Definir los pasos de un procedimiento</t>
+        </is>
+      </c>
+      <c r="D340" s="10" t="inlineStr">
+        <is>
+          <t>API_UPD_ORDEN_TRABAJO_PASO (bloque 244): un paso que exige medición no se completa sin el valor y lo registra en Activo_Medicion con la OT como origen (#2); un punto de control pendiente bloquea los pasos siguientes (#3).</t>
+        </is>
+      </c>
+      <c r="E340" s="6" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
+      <c r="F340" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G340" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="H340" s="6" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I340" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J340" s="7" t="inlineStr">
+        <is>
+          <t>Construido y probado el 17-09-2026 (evidencia S3 por criterio). Tomado por Bryan a pedido suyo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="15.75" customHeight="1" s="19">
+      <c r="A341" s="6" t="inlineStr">
+        <is>
+          <t>T-3977</t>
+        </is>
+      </c>
+      <c r="B341" s="6" t="inlineStr">
+        <is>
+          <t>HU-062</t>
+        </is>
+      </c>
+      <c r="C341" s="7" t="inlineStr">
+        <is>
+          <t>Definir los pasos de un procedimiento</t>
+        </is>
+      </c>
+      <c r="D341" s="10" t="inlineStr">
+        <is>
+          <t>PasoResultadoDto gana valor_medicion y unidad_medida; el controller los pasa al SP. Compila 0 errores.</t>
+        </is>
+      </c>
+      <c r="E341" s="6" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F341" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G341" s="7" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="H341" s="6" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I341" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J341" s="7" t="inlineStr">
+        <is>
+          <t>Construido y probado el 17-09-2026 (evidencia S3 por criterio). Tomado por Bryan a pedido suyo.</t>
+        </is>
+      </c>
+    </row>
     <row r="342" ht="15.75" customHeight="1" s="19"/>
     <row r="343" ht="15.75" customHeight="1" s="19"/>
     <row r="344" ht="15.75" customHeight="1" s="19"/>
@@ -21420,7 +21702,7 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -21453,7 +21735,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22658,7 +22940,7 @@
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22784,7 +23066,7 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22816,7 +23098,7 @@
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22847,7 +23129,7 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22974,7 +23256,7 @@
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -23005,7 +23287,7 @@
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>

</xml_diff>